<commit_message>
sp_ui: add manual_triage_required column for FR-12 path (c.2) below-threshold triage
Inserts manual_triage_required BOOLEAN column at row 48 of DI field
visibility tab (immediately after last_owner_response_at and before
doc_count). Default = FALSE.

Set to TRUE by HILDA when an inbound owner reply (per FR-12) fails
the rule-based + LLM classification below confidence threshold —
surfaces a Manual triage flag on the PM dashboard for TPM resolution.
TPM clears (sets to FALSE) when triage is resolved (after reading the
original email + writing the correct delivery_state per FR-14).

Column attributes:
- Display class: must_show (PM dashboard surfaces the triage queue)
- Writable in SP UI: YES (TPM)
- SP UI engineer modifies in code: NO
- SP UI engineer reads in code: YES (to surface triage queue +
  allow TPM-clear action)

Closes the xlsx column add pending from FR-12 review commit d9601db.
</commit_message>
<xml_diff>
--- a/docs/sp_ui_engineer/SP_lists_authoritative.xlsx
+++ b/docs/sp_ui_engineer/SP_lists_authoritative.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1008"/>
+  <dimension ref="A1:H1009"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="47" customWidth="1" style="35" min="1" max="1"/>
@@ -2237,22 +2237,22 @@
     <row r="48" ht="17.25" customHeight="1" s="35">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>doc_count</t>
+          <t>manual_triage_required</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>not_to_be_shown</t>
+          <t>must_show</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES (TPM)</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -2262,24 +2262,24 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G48" s="21" t="inlineStr">
-        <is>
-          <t>for hilda purposes only</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G48" s="36" t="inlineStr">
+        <is>
+          <t>HILDA-managed boolean column. Default = FALSE. Set to TRUE by HILDA when an inbound owner reply (per FR-12) fails the rule-based + LLM classification below confidence threshold — surfaces a Manual triage flag on the PM dashboard. TPM clears (sets to FALSE) when triage is resolved (after reading the original email and writing the correct delivery_state per FR-14). SP UI engineer reads this column to surface the triage queue in the PM dashboard; SP UI engineer's web part allows TPM to clear the flag once resolved.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1" s="35">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>review_status</t>
+          <t>doc_count</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>LIST</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -2304,19 +2304,19 @@
       </c>
       <c r="G49" s="21" t="inlineStr">
         <is>
-          <t>(pending / complete / not_required); for hilda purposes only</t>
+          <t>for hilda purposes only</t>
         </is>
       </c>
     </row>
     <row r="50" ht="17.25" customHeight="1" s="35">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>ingress_folder</t>
+          <t>review_status</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>LIST</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -2339,16 +2339,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G50" s="18" t="inlineStr">
-        <is>
-          <t>for hilda purposes only; e.g. \carrierX\deviceY\milestoneZ\WiFi_Conformance\</t>
+      <c r="G50" s="21" t="inlineStr">
+        <is>
+          <t>(pending / complete / not_required); for hilda purposes only</t>
         </is>
       </c>
     </row>
     <row r="51" ht="21" customHeight="1" s="35">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>target_folder</t>
+          <t>ingress_folder</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
@@ -2376,21 +2376,21 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
-        <is>
-          <t>for hilda purposes only; e.g. drive.google.com\vzw\SM-S901U</t>
+      <c r="G51" s="18" t="inlineStr">
+        <is>
+          <t>for hilda purposes only; e.g. \carrierX\deviceY\milestoneZ\WiFi_Conformance\</t>
         </is>
       </c>
     </row>
     <row r="52" ht="20.25" customHeight="1" s="35">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>pm_approval_at</t>
+          <t>target_folder</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>DATE/TIME</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -2403,9 +2403,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -2413,21 +2413,21 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G52" s="18" t="inlineStr">
-        <is>
-          <t>When TPM approves a work item, SP UI engineer updates this field</t>
+      <c r="G52" s="22" t="inlineStr">
+        <is>
+          <t>for hilda purposes only; e.g. drive.google.com\vzw\SM-S901U</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18.75" customHeight="1" s="35">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>pm_approval_pm_id</t>
+          <t>pm_approval_at</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>DATE/TIME</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -2459,12 +2459,12 @@
     <row r="54" ht="32.25" customHeight="1" s="35">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>tpm_reassignment_target_item_id</t>
+          <t>pm_approval_pm_id</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -2477,9 +2477,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -2489,19 +2489,19 @@
       </c>
       <c r="G54" s="18" t="inlineStr">
         <is>
-          <t>for hilda internal purposes only; resets work-item id of a document;</t>
+          <t>When TPM approves a work item, SP UI engineer updates this field</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="35">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>tpm_resolved_doc_type</t>
+          <t>tpm_reassignment_target_item_id</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -2526,14 +2526,14 @@
       </c>
       <c r="G55" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">for hilda internal purposes only; resolves document type of a document; </t>
+          <t>for hilda internal purposes only; resets work-item id of a document;</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="35">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>tpm_revision_resolution</t>
+          <t>tpm_resolved_doc_type</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
@@ -2563,132 +2563,132 @@
       </c>
       <c r="G56" s="18" t="inlineStr">
         <is>
-          <t>for hilda internal purposes only; resolves new/revised revision of a document;</t>
+          <t xml:space="preserve">for hilda internal purposes only; resolves document type of a document; </t>
         </is>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="35">
       <c r="A57" s="11" t="inlineStr">
         <is>
+          <t>tpm_revision_resolution</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>not_to_be_shown</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>for hilda internal purposes only; resolves new/revised revision of a document;</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
           <t>ingress_nsd (denorm TG)</t>
         </is>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B58" s="11" t="inlineStr">
         <is>
           <t>LIST</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G57" s="18" t="inlineStr">
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="inlineStr">
         <is>
           <t>list values: NSD1, NSD2, none
 (two different network shared drives that different TGs use)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="59" ht="15.75" customHeight="1" s="35">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>list_documents_url_prefix (ideal storage
  is in SP Java script config, not here)</t>
         </is>
       </c>
-      <c r="B58" s="11" t="inlineStr">
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F58" s="8" t="inlineStr">
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="G58" s="20" t="inlineStr">
+      <c r="G59" s="20" t="inlineStr">
         <is>
           <t>SP constructs docs URL with list_documents_url_prefix/item_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="15.75" customHeight="1" s="35">
-      <c r="A59" s="11" t="inlineStr">
-        <is>
-          <t>folder_routing_enabled (denorm)</t>
-        </is>
-      </c>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>BOOL</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>not_to_be_shown</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G59" s="36" t="inlineStr">
-        <is>
-          <t>hilda internal purposes; TGs using network shared drives to deliver documents</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="35">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>per_item_rule_overrides</t>
+          <t>folder_routing_enabled (denorm)</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>STR</t>
+          <t>BOOL</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2713,112 +2713,112 @@
       </c>
       <c r="G60" s="36" t="inlineStr">
         <is>
-          <t>for hilda purposes only; Ph-2 placeholder - August 1' 2026 delivery.</t>
+          <t>hilda internal purposes; TGs using network shared drives to deliver documents</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="35">
       <c r="A61" s="11" t="inlineStr">
         <is>
+          <t>per_item_rule_overrides</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>not_to_be_shown</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G61" s="36" t="inlineStr">
+        <is>
+          <t>for hilda purposes only; Ph-2 placeholder - August 1' 2026 delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1" s="35">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
           <t>sort_order</t>
         </is>
       </c>
-      <c r="B61" s="11" t="n"/>
-      <c r="C61" s="23" t="inlineStr">
+      <c r="B62" s="11" t="n"/>
+      <c r="C62" s="23" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G61" s="36" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G62" s="36" t="inlineStr">
         <is>
           <t>Controls display order; not a visible column</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="15.75" customHeight="1" s="35">
-      <c r="A62" s="25" t="n"/>
-      <c r="B62" s="11" t="n"/>
-      <c r="C62" s="25" t="n"/>
-      <c r="D62" s="25" t="n"/>
-      <c r="E62" s="34" t="n"/>
-      <c r="F62" s="34" t="n"/>
-      <c r="G62" s="34" t="n"/>
-    </row>
     <row r="63" ht="15.75" customHeight="1" s="35">
-      <c r="A63" s="27" t="inlineStr">
+      <c r="A63" s="25" t="n"/>
+      <c r="B63" s="11" t="n"/>
+      <c r="C63" s="25" t="n"/>
+      <c r="D63" s="25" t="n"/>
+      <c r="E63" s="34" t="n"/>
+      <c r="F63" s="34" t="n"/>
+      <c r="G63" s="34" t="n"/>
+    </row>
+    <row r="64" ht="15.75" customHeight="1" s="35">
+      <c r="A64" s="27" t="inlineStr">
         <is>
           <t>Milestone SP List
 * clean separation from delivery items, avoid hacks</t>
         </is>
       </c>
-      <c r="B63" s="29" t="n"/>
-      <c r="C63" s="29" t="n"/>
-      <c r="D63" s="29" t="n"/>
-      <c r="E63" s="20" t="n"/>
-      <c r="F63" s="20" t="n"/>
-      <c r="G63" s="20" t="n"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1" s="35">
-      <c r="A64" s="29" t="inlineStr">
-        <is>
-          <t>milestone_id</t>
-        </is>
-      </c>
-      <c r="B64" s="11" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="C64" s="14" t="inlineStr">
-        <is>
-          <t>must_show</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F64" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G64" s="20" t="inlineStr">
-        <is>
-          <t>primary key</t>
-        </is>
-      </c>
+      <c r="B64" s="29" t="n"/>
+      <c r="C64" s="29" t="n"/>
+      <c r="D64" s="29" t="n"/>
+      <c r="E64" s="20" t="n"/>
+      <c r="F64" s="20" t="n"/>
+      <c r="G64" s="20" t="n"/>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="35">
       <c r="A65" s="29" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>milestone_id</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>LIST</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
@@ -2836,106 +2836,106 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F65" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="G65" s="20" t="inlineStr">
         <is>
-          <t>list-values {Not Started, In Progress, Completed, Delayed}, SP engineer uses this to check if start collection button to be displayed in milestone view</t>
+          <t>primary key</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="35">
       <c r="A66" s="29" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>LIST</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>must_show</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G66" s="20" t="inlineStr">
+        <is>
+          <t>list-values {Not Started, In Progress, Completed, Delayed}, SP engineer uses this to check if start collection button to be displayed in milestone view</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1" s="35">
+      <c r="A67" s="29" t="inlineStr">
+        <is>
           <t>download_package_request_timestamp</t>
         </is>
       </c>
-      <c r="B66" s="11" t="inlineStr">
+      <c r="B67" s="11" t="inlineStr">
         <is>
           <t>DATE/TIME</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D66" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F66" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G66" s="20" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G67" s="20" t="inlineStr">
         <is>
           <t>SP engineer writes when TPM clicks Download Package button.
 The act of writing this field is what fires the SP-alert email</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1" s="35">
-      <c r="A67" s="29" t="inlineStr">
-        <is>
-          <t>download_package_status</t>
-        </is>
-      </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>LIST</t>
-        </is>
-      </c>
-      <c r="C67" s="14" t="inlineStr">
-        <is>
-          <t>must_show</t>
-        </is>
-      </c>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F67" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="G67" s="20" t="inlineStr">
-        <is>
-          <t>HILDA-write. Enum: preparing | ready | failed. Set to preparing immediately by SP UI on click (mirror of request_timestamp); HILDA writes ready on assembly success / failed on assembly error. SP web part reads this on focus-aware refresh to decide whether to show "Preparing..." indicator or Download Now link</t>
-        </is>
-      </c>
-    </row>
     <row r="68" ht="15.75" customHeight="1" s="35">
       <c r="A68" s="29" t="inlineStr">
         <is>
-          <t>download_package_url</t>
+          <t>download_package_status</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>STR</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>not_to_be_shown</t>
+          <t>LIST</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>must_show</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -2943,9 +2943,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -2955,19 +2955,19 @@
       </c>
       <c r="G68" s="20" t="inlineStr">
         <is>
-          <t>HILDA-write. The scoped download URL https://hilda-proxy.corp/dl/&lt;scoped_token&gt; HILDA generates when assembly succeeds. The clickable target of the Download Now link. Null until status=ready</t>
+          <t>HILDA-write. Enum: preparing | ready | failed. Set to preparing immediately by SP UI on click (mirror of request_timestamp); HILDA writes ready on assembly success / failed on assembly error. SP web part reads this on focus-aware refresh to decide whether to show "Preparing..." indicator or Download Now link</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="35">
       <c r="A69" s="29" t="inlineStr">
         <is>
-          <t>download_package_generated_at</t>
+          <t>download_package_url</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>DATE/TIME</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -2985,21 +2985,21 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="G69" s="20" t="inlineStr">
         <is>
-          <t>HILDA-write. Timestamp of assembly completion; used for cache-staleness display ("generated 3 min ago")</t>
+          <t>HILDA-write. The scoped download URL https://hilda-proxy.corp/dl/&lt;scoped_token&gt; HILDA generates when assembly succeeds. The clickable target of the Download Now link. Null until status=ready</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="35">
       <c r="A70" s="29" t="inlineStr">
         <is>
-          <t>milestone_collection_started_at</t>
+          <t>download_package_generated_at</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
@@ -3017,26 +3017,26 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="G70" s="20" t="inlineStr">
         <is>
-          <t>SP engineer uses this to check if start collection button to be displayed in milestone view. SP engineer modifies this field once collection started. The act of writing this field is what fires the SP-alert email</t>
+          <t>HILDA-write. Timestamp of assembly completion; used for cache-staleness display ("generated 3 min ago")</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="35">
       <c r="A71" s="29" t="inlineStr">
         <is>
-          <t>milestone_submission_triggered_at</t>
+          <t>milestone_collection_started_at</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
@@ -3059,256 +3059,284 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="G71" s="20" t="inlineStr">
         <is>
-          <t>SP engineer modifies this field once submit to carrier button is clicked. The act of writing this field is what fires the SP-alert email</t>
+          <t>SP engineer uses this to check if start collection button to be displayed in milestone view. SP engineer modifies this field once collection started. The act of writing this field is what fires the SP-alert email</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="35">
       <c r="A72" s="29" t="inlineStr">
         <is>
-          <t>target_date</t>
+          <t>milestone_submission_triggered_at</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>DATE</t>
-        </is>
-      </c>
-      <c r="C72" s="14" t="inlineStr">
-        <is>
-          <t>must_show</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
+          <t>DATE/TIME</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>not_to_be_shown</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F72" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="G72" s="20" t="inlineStr">
         <is>
-          <t>update expected_completion_date of all delivery items / work items of this milestone. The act of writing this field is what fires the SP-alert email</t>
+          <t>SP engineer modifies this field once submit to carrier button is clicked. The act of writing this field is what fires the SP-alert email</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="35">
       <c r="A73" s="29" t="inlineStr">
         <is>
-          <t>refresh_requested_at</t>
+          <t>target_date</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>DATE/TIME</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>not_to_be_shown</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>must_show</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="G73" s="20" t="inlineStr">
         <is>
-          <t>SP engineer modifies this field once refresh button is clicked. The act of writing this field is what fires the SP-alert email</t>
+          <t>update expected_completion_date of all delivery items / work items of this milestone. The act of writing this field is what fires the SP-alert email</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1" s="35">
       <c r="A74" s="29" t="inlineStr">
         <is>
+          <t>refresh_requested_at</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>DATE/TIME</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>not_to_be_shown</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G74" s="20" t="inlineStr">
+        <is>
+          <t>SP engineer modifies this field once refresh button is clicked. The act of writing this field is what fires the SP-alert email</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15.75" customHeight="1" s="35">
+      <c r="A75" s="29" t="inlineStr">
+        <is>
           <t>closed_all_items_triggered_at</t>
         </is>
       </c>
-      <c r="B74" s="11" t="inlineStr">
+      <c r="B75" s="11" t="inlineStr">
         <is>
           <t>DATE/TIME</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D74" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F74" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G74" s="20" t="inlineStr">
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G75" s="20" t="inlineStr">
         <is>
           <t>SP engineer modifies this field once close all items button is clicked. The act of writing this field is what fires the SP-alert email</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="15.75" customHeight="1" s="35">
-      <c r="A75" s="25" t="n"/>
-      <c r="B75" s="25" t="n"/>
-      <c r="C75" s="25" t="n"/>
-      <c r="D75" s="25" t="n"/>
-      <c r="E75" s="30" t="n"/>
-      <c r="F75" s="30" t="n"/>
-      <c r="G75" s="30" t="n"/>
-    </row>
     <row r="76" ht="15.75" customHeight="1" s="35">
-      <c r="A76" s="31" t="inlineStr">
+      <c r="A76" s="25" t="n"/>
+      <c r="B76" s="25" t="n"/>
+      <c r="C76" s="25" t="n"/>
+      <c r="D76" s="25" t="n"/>
+      <c r="E76" s="30" t="n"/>
+      <c r="F76" s="30" t="n"/>
+      <c r="G76" s="30" t="n"/>
+    </row>
+    <row r="77" ht="15.75" customHeight="1" s="35">
+      <c r="A77" s="31" t="inlineStr">
         <is>
           <t>Customer SP list (need not be a new list, 
 need below values from customer_id)</t>
         </is>
       </c>
-      <c r="B76" s="29" t="n"/>
-      <c r="C76" s="29" t="n"/>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="32" t="n"/>
-      <c r="F76" s="32" t="n"/>
-      <c r="G76" s="32" t="n"/>
-    </row>
-    <row r="77" ht="15.75" customHeight="1" s="35">
-      <c r="A77" s="29" t="inlineStr">
+      <c r="B77" s="29" t="n"/>
+      <c r="C77" s="29" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="32" t="n"/>
+      <c r="F77" s="32" t="n"/>
+      <c r="G77" s="32" t="n"/>
+    </row>
+    <row r="78" ht="15.75" customHeight="1" s="35">
+      <c r="A78" s="29" t="inlineStr">
         <is>
           <t>customer_jira_url</t>
         </is>
       </c>
-      <c r="B77" s="11" t="inlineStr">
+      <c r="B78" s="11" t="inlineStr">
         <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C78" s="6" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E77" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G77" s="20" t="inlineStr">
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G78" s="20" t="inlineStr">
         <is>
           <t>hilda internal purposes only</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="15.75" customHeight="1" s="35">
-      <c r="A78" s="33" t="n"/>
-      <c r="B78" s="33" t="n"/>
-      <c r="C78" s="33" t="n"/>
-      <c r="D78" s="33" t="n"/>
-      <c r="E78" s="33" t="n"/>
-      <c r="F78" s="33" t="n"/>
-      <c r="G78" s="33" t="n"/>
-    </row>
     <row r="79" ht="15.75" customHeight="1" s="35">
-      <c r="A79" s="31" t="inlineStr">
+      <c r="A79" s="33" t="n"/>
+      <c r="B79" s="33" t="n"/>
+      <c r="C79" s="33" t="n"/>
+      <c r="D79" s="33" t="n"/>
+      <c r="E79" s="33" t="n"/>
+      <c r="F79" s="33" t="n"/>
+      <c r="G79" s="33" t="n"/>
+    </row>
+    <row r="80" ht="15.75" customHeight="1" s="35">
+      <c r="A80" s="31" t="inlineStr">
         <is>
           <t>Devices SP list (need not be a new list,
 need below value from device_id)</t>
         </is>
       </c>
-      <c r="B79" s="29" t="n"/>
-      <c r="C79" s="29" t="n"/>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="32" t="n"/>
-      <c r="F79" s="32" t="n"/>
-      <c r="G79" s="32" t="n"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1" s="35">
-      <c r="A80" s="29" t="inlineStr">
+      <c r="B80" s="29" t="n"/>
+      <c r="C80" s="29" t="n"/>
+      <c r="D80" s="29" t="n"/>
+      <c r="E80" s="32" t="n"/>
+      <c r="F80" s="32" t="n"/>
+      <c r="G80" s="32" t="n"/>
+    </row>
+    <row r="81" ht="15.75" customHeight="1" s="35">
+      <c r="A81" s="29" t="inlineStr">
         <is>
           <t>assigned_pm_id (SEA email address of TPM)</t>
         </is>
       </c>
-      <c r="B80" s="11" t="inlineStr">
+      <c r="B81" s="11" t="inlineStr">
         <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="C80" s="6" t="inlineStr">
+      <c r="C81" s="6" t="inlineStr">
         <is>
           <t>not_to_be_shown</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E80" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F80" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G80" s="20" t="inlineStr">
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G81" s="20" t="inlineStr">
         <is>
           <t>hilda internal purposes only</t>
         </is>
       </c>
-    </row>
-    <row r="81" ht="15.75" customHeight="1" s="35">
-      <c r="A81" s="25" t="n"/>
-      <c r="B81" s="25" t="n"/>
-      <c r="C81" s="25" t="n"/>
-      <c r="D81" s="25" t="n"/>
-      <c r="E81" s="34" t="n"/>
-      <c r="F81" s="34" t="n"/>
-      <c r="G81" s="34" t="n"/>
     </row>
     <row r="82" ht="15.75" customHeight="1" s="35">
       <c r="A82" s="25" t="n"/>
@@ -3319,16 +3347,16 @@
       <c r="F82" s="34" t="n"/>
       <c r="G82" s="34" t="n"/>
     </row>
-    <row r="83" ht="15.75" customHeight="1" s="35"/>
-    <row r="84" ht="15.75" customHeight="1" s="35">
-      <c r="A84" s="25" t="n"/>
-      <c r="B84" s="25" t="n"/>
-      <c r="C84" s="25" t="n"/>
-      <c r="D84" s="25" t="n"/>
-      <c r="E84" s="34" t="n"/>
-      <c r="F84" s="34" t="n"/>
-      <c r="G84" s="34" t="n"/>
-    </row>
+    <row r="83" ht="15.75" customHeight="1" s="35">
+      <c r="A83" s="25" t="n"/>
+      <c r="B83" s="25" t="n"/>
+      <c r="C83" s="25" t="n"/>
+      <c r="D83" s="25" t="n"/>
+      <c r="E83" s="34" t="n"/>
+      <c r="F83" s="34" t="n"/>
+      <c r="G83" s="34" t="n"/>
+    </row>
+    <row r="84" ht="15.75" customHeight="1" s="35"/>
     <row r="85" ht="15.75" customHeight="1" s="35">
       <c r="A85" s="25" t="n"/>
       <c r="B85" s="25" t="n"/>
@@ -11645,6 +11673,15 @@
       <c r="F1008" s="34" t="n"/>
       <c r="G1008" s="34" t="n"/>
     </row>
+    <row r="1009">
+      <c r="A1009" s="25" t="n"/>
+      <c r="B1009" s="25" t="n"/>
+      <c r="C1009" s="25" t="n"/>
+      <c r="D1009" s="25" t="n"/>
+      <c r="E1009" s="34" t="n"/>
+      <c r="F1009" s="34" t="n"/>
+      <c r="G1009" s="34" t="n"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId1"/>

</xml_diff>

<commit_message>
xlsx: add column H "LIST values (Choice enums)" for SP-provisioning reference
Populated for 10 LIST-type rows:
- item_type (4 values per FR-7)
- delivery_state (11 values per FR-7)
- prior_delivery_state (same 11 as delivery_state)
- tracking_modality (6 values per FR-7; multi-select)
- tg_name (per-customer; template.yaml-driven)
- customer_delivery_modality (TBD — architect confirmation at provision time)
- review_status (pending / complete / failed per FR-53/FR-62/FR-87)
- ingress_nsd (none / nsd1 / nsd2 per FR-13)
- status (Milestones; 4 values per FR-6 precedence ladder)
- download_package_status (preparing / ready / failed per FR-73 [Ph-2])

Closes STATUS Flag: Sheet Choice value verifications.

Open follow-up: customer_delivery_modality enum needs architect lock
(currently observed test samples: Email, CustomerTrackingSystem) —
architect to confirm full set at SP-list provisioning time.
</commit_message>
<xml_diff>
--- a/docs/sp_ui_engineer/SP_lists_authoritative.xlsx
+++ b/docs/sp_ui_engineer/SP_lists_authoritative.xlsx
@@ -595,7 +595,11 @@
           <t>Notes for SP UI Engineer</t>
         </is>
       </c>
-      <c r="H1" s="5" t="n"/>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>LIST values (Choice enums)</t>
+        </is>
+      </c>
       <c r="I1" s="5" t="n"/>
       <c r="J1" s="5" t="n"/>
       <c r="K1" s="5" t="n"/>
@@ -1130,7 +1134,11 @@
 delivery_item_type : what type of document being delivered</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Confirmation, TEST_TECH_WAIVER_REPORT, COMPLIANCE_CERTIFICATION_RELEASE_NOTES, Default (4 values per FR-7)</t>
+        </is>
+      </c>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
@@ -1186,7 +1194,11 @@
           <t>11-value Choice (Not Started, Open, OutreachSent, DocumentReceived, UnderPMReview, OwnerClosed, Delayed, Blocked, ReadyForSubmission, SubmittedToCustomer, Closed). list-value = 'Not Started' is SP-side state for TPM-loaded-template-not-yet-started-tracking; SP UI engineer uses this field to show start collection button, close all items button in milestone view, display approve button, send reminder button, documents button in per-work-item view. WRITABLE BY TPM via cell-edit (per FR-14 + FR-56 I2 lock 2026-06-16) — but RESERVED for two residual use cases only: (1) setting Delayed/Blocked from an active state when TPM observes external delay/blocker before owner reports; (2) rolling back an erroneously-fired automated transition (e.g., wrongly-advanced ReadyForSubmission). All OTHER state changes go via dedicated per-row buttons (Approve, Mark Closed, Confirm Carrier Acceptance, Resume from Delayed/Blocked) per SP_UI_button_actions.md Part 1. HILDA's sp_alert_parser auto-manages prior_delivery_state per FR-7 I2 / FR-12 / FR-14 discipline on Delayed/Blocked transitions.</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n"/>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Not Started, Open, OutreachSent, DocumentReceived, UnderPMReview, OwnerClosed, Delayed, Blocked, ReadyForSubmission, SubmittedToCustomer, Closed (11 values per FR-7 — SP-only Not Started + 10 HILDA enum values)</t>
+        </is>
+      </c>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="n"/>
@@ -1242,7 +1254,11 @@
           <t>Same 11-value Choice enum as delivery_state. HILDA-written audit column: stores the state immediately preceding entry into 'Delayed' or 'Blocked'; set by HILDA when transitioning into Delayed/Blocked; cleared (set to NULL) when transitioning out. Enables HILDA to restore the prior active state on exit per FR-7. SP UI engineer does NOT read or write this column.</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Same 11 values as delivery_state per FR-7 (HILDA-written; SP UI engineer does not read or write)</t>
+        </is>
+      </c>
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="5" t="n"/>
       <c r="K13" s="5" t="n"/>
@@ -1850,7 +1866,11 @@
           <t>MultiChoice {Email, CorporateMessenger, CorporatePLM, NetworkSharedDrive, Customer JIRA, SPUI} ]</t>
         </is>
       </c>
-      <c r="H24" s="5" t="n"/>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Email, CorporateMessenger, CorporatePLM, NetworkSharedDrive, CustomerJIRA, SPUI (6 values per FR-7; multi-select)</t>
+        </is>
+      </c>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
       <c r="K24" s="5" t="n"/>
@@ -2010,7 +2030,11 @@
           <t>enum {SW PL, HW PL, CPM, MNO-UX, MNO-TPM, MNO-ETM, MNO-IOT, MNO-SOLUTION, MNO-OMADM, MQL-FIT, MQL, MQL PC, GPS, MNO-SELNA, APPS, MNO-DTR}</t>
         </is>
       </c>
-      <c r="H27" s="5" t="n"/>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Per-customer; values set by template.yaml TG definitions per FR-40 (no fixed enum across customers)</t>
+        </is>
+      </c>
       <c r="I27" s="5" t="n"/>
       <c r="J27" s="5" t="n"/>
       <c r="K27" s="5" t="n"/>
@@ -2927,7 +2951,11 @@
           <t>values {GoogleDrive, Email, Customer tracking system}; type of system to which documents are uploaded</t>
         </is>
       </c>
-      <c r="H44" s="5" t="n"/>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>TBD — confirm with architect at SP-list-provisioning time (observed test sample: Email, CustomerTrackingSystem)</t>
+        </is>
+      </c>
       <c r="I44" s="5" t="n"/>
       <c r="J44" s="5" t="n"/>
       <c r="K44" s="5" t="n"/>
@@ -3376,7 +3404,11 @@
           <t>4-value Choice enum: (pending / complete / not_required / failed). HILDA-managed; for HILDA purposes only — not shown in SP UI. Lifecycle per FR-53 I14/I15: pending = at least one received doc has review not yet complete (default at row creation when review_required=true); complete = ALL received docs reviewed (each DocumentIndexRow.llm_review_findings non-null) — required to satisfy FR-7 OwnerClosed guard condition (2) for items passing through OwnerClosed; not_required = review_required=false on item; failed = at least one received doc has persistent LLM review failure (added 2026-06-16 per FR-53 I8). SP UI engineer does NOT read or write this column.</t>
         </is>
       </c>
-      <c r="H52" s="5" t="n"/>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>pending, complete, failed (3 values per FR-53 / FR-62 / FR-87 lifecycle)</t>
+        </is>
+      </c>
       <c r="I52" s="5" t="n"/>
       <c r="J52" s="5" t="n"/>
       <c r="K52" s="5" t="n"/>
@@ -3825,7 +3857,11 @@
 (two different network shared drives that different TGs use)  (denorm TG)</t>
         </is>
       </c>
-      <c r="H60" s="5" t="n"/>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>none, nsd1, nsd2 (3 values per FR-13 flat per-TG folder structure)</t>
+        </is>
+      </c>
       <c r="I60" s="5" t="n"/>
       <c r="J60" s="5" t="n"/>
       <c r="K60" s="5" t="n"/>
@@ -4511,7 +4547,11 @@
           <t>list-values {Not Started, In Progress, Completed, Delayed}, SP engineer uses this to check if start collection button to be displayed in milestone view</t>
         </is>
       </c>
-      <c r="H74" s="5" t="n"/>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Not Started, In Progress, Completed, Delayed (4 values per FR-6 precedence ladder)</t>
+        </is>
+      </c>
       <c r="I74" s="5" t="n"/>
       <c r="J74" s="5" t="n"/>
       <c r="K74" s="5" t="n"/>
@@ -4624,7 +4664,11 @@
           <t>HILDA-write. Enum: preparing | ready | failed. Set to preparing immediately by SP UI on click (mirror of request_timestamp); HILDA writes ready on assembly success / failed on assembly error. SP web part reads this on focus-aware refresh to decide whether to show "Preparing..." indicator or Download Now link</t>
         </is>
       </c>
-      <c r="H76" s="5" t="n"/>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>preparing, ready, failed (3 values per FR-73; [Ph-2] deferred)</t>
+        </is>
+      </c>
       <c r="I76" s="5" t="n"/>
       <c r="J76" s="5" t="n"/>
       <c r="K76" s="5" t="n"/>

</xml_diff>